<commit_message>
Changes made to integrate model tuning
</commit_message>
<xml_diff>
--- a/datasets/current_points_table.xlsx
+++ b/datasets/current_points_table.xlsx
@@ -467,28 +467,28 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I2" t="n">
         <v>1</v>
@@ -496,28 +496,28 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I3" t="n">
         <v>2</v>
@@ -525,28 +525,28 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I4" t="n">
         <v>3</v>
@@ -554,7 +554,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B5" t="n">
         <v>0</v>
@@ -563,19 +563,19 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I5" t="n">
         <v>4</v>
@@ -583,28 +583,28 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B6" t="n">
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I6" t="n">
         <v>5</v>
@@ -612,28 +612,28 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B7" t="n">
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I7" t="n">
         <v>6</v>
@@ -641,7 +641,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B8" t="n">
         <v>0</v>
@@ -650,19 +650,19 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I8" t="n">
         <v>7</v>
@@ -670,28 +670,28 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I9" t="n">
         <v>8</v>
@@ -699,28 +699,28 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I10" t="n">
         <v>9</v>
@@ -728,28 +728,28 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I11" t="n">
         <v>10</v>
@@ -757,28 +757,28 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I12" t="n">
         <v>11</v>
@@ -786,28 +786,28 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I13" t="n">
         <v>12</v>
@@ -815,28 +815,28 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B14" t="n">
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I14" t="n">
         <v>13</v>
@@ -844,28 +844,28 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15" t="n">
         <v>14</v>
@@ -873,28 +873,28 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I16" t="n">
         <v>15</v>
@@ -902,28 +902,28 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I17" t="n">
         <v>16</v>
@@ -931,28 +931,28 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I18" t="n">
         <v>17</v>
@@ -960,28 +960,28 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I19" t="n">
         <v>18</v>
@@ -992,25 +992,25 @@
         <v>0</v>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C20" t="n">
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I20" t="n">
         <v>19</v>
@@ -1021,25 +1021,25 @@
         <v>0</v>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21" t="n">
         <v>20</v>
@@ -1112,13 +1112,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -1127,16 +1127,16 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J2" t="n">
         <v>1</v>
@@ -1144,31 +1144,31 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J3" t="n">
         <v>2</v>
@@ -1176,31 +1176,31 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
@@ -1208,31 +1208,31 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B5" t="n">
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J5" t="n">
         <v>4</v>
@@ -1240,31 +1240,31 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="B6" t="n">
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J6" t="n">
         <v>5</v>
@@ -1272,31 +1272,31 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="B7" t="n">
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J7" t="n">
         <v>6</v>
@@ -1304,31 +1304,31 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B8" t="n">
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J8" t="n">
         <v>7</v>
@@ -1336,31 +1336,31 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J9" t="n">
         <v>8</v>
@@ -1368,31 +1368,31 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J10" t="n">
         <v>9</v>
@@ -1400,31 +1400,31 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
+        <v>10</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>12</v>
+      </c>
+      <c r="G11" t="n">
         <v>6</v>
       </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J11" t="n">
         <v>10</v>
@@ -1432,31 +1432,31 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
+        <v>11</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>11</v>
+      </c>
+      <c r="G12" t="n">
         <v>10</v>
       </c>
-      <c r="E12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
-      </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J12" t="n">
         <v>11</v>
@@ -1464,31 +1464,31 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J13" t="n">
         <v>12</v>
@@ -1496,31 +1496,31 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J14" t="n">
         <v>13</v>
@@ -1528,31 +1528,31 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J15" t="n">
         <v>14</v>
@@ -1560,31 +1560,31 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J16" t="n">
         <v>15</v>
@@ -1592,31 +1592,31 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J17" t="n">
         <v>16</v>
@@ -1624,31 +1624,31 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J18" t="n">
         <v>17</v>
@@ -1656,31 +1656,31 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B19" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J19" t="n">
         <v>18</v>
@@ -1688,31 +1688,31 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C20" t="n">
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J20" t="n">
         <v>19</v>
@@ -1720,31 +1720,31 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J21" t="n">
         <v>20</v>
@@ -1793,22 +1793,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>Manchester City</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>43</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>Man City</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ARS</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1818,22 +1818,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Manchester City</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Man City</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>ARS</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1843,22 +1843,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Manchester United</t>
+          <t>Brighton and Hove Albion</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>36</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Man Utd</t>
+          <t>Brighton</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MUN</t>
+          <t>BHA</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1868,22 +1868,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Aston Villa</t>
+          <t>Brentford</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>94</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Aston Villa</t>
+          <t>Brentford</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>AVL</t>
+          <t>BRE</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1893,22 +1893,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>Leeds United</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>Leeds</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>LIV</t>
+          <t>LEE</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1918,22 +1918,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Bournemouth</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Bournemouth</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>BOU</t>
+          <t>LIV</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1943,22 +1943,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sunderland</t>
+          <t>Everton</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sunderland</t>
+          <t>Everton</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SUN</t>
+          <t>EVE</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -1968,22 +1968,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Brighton and Hove Albion</t>
+          <t>Hull City</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>88</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Brighton</t>
+          <t>Hull</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>BHA</t>
+          <t>HUL</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1993,22 +1993,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Brentford</t>
+          <t>Newcastle United</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Brentford</t>
+          <t>Newcastle</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>BRE</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -2043,22 +2043,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Fulham</t>
+          <t>Ipswich Town</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fulham</t>
+          <t>Ipswich</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FUL</t>
+          <t>IPS</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -2068,22 +2068,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Newcastle United</t>
+          <t>Manchester United</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Newcastle</t>
+          <t>Man Utd</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>MUN</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -2093,22 +2093,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Everton</t>
+          <t>Nottingham Forest</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Everton</t>
+          <t>Nott'm Forest</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>EVE</t>
+          <t>NFO</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -2118,22 +2118,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Leeds United</t>
+          <t>Sunderland</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>56</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Leeds</t>
+          <t>Sunderland</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>LEE</t>
+          <t>SUN</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -2168,22 +2168,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Nottingham Forest</t>
+          <t>Aston Villa</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Nott'm Forest</t>
+          <t>Aston Villa</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>NFO</t>
+          <t>AVL</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -2193,22 +2193,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Tottenham Hotspur</t>
+          <t>Bournemouth</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>91</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Spurs</t>
+          <t>Bournemouth</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>TOT</t>
+          <t>BOU</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -2243,22 +2243,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ipswich Town</t>
+          <t>Fulham</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>54</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ipswich</t>
+          <t>Fulham</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>IPS</t>
+          <t>FUL</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -2268,22 +2268,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Hull City</t>
+          <t>Tottenham Hotspur</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Hull</t>
+          <t>Spurs</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>HUL</t>
+          <t>TOT</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -2352,13 +2352,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -2367,13 +2367,13 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I2" t="n">
         <v>1</v>
@@ -2381,28 +2381,28 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B3" t="n">
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I3" t="n">
         <v>2</v>
@@ -2410,28 +2410,28 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="B4" t="n">
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I4" t="n">
         <v>3</v>
@@ -2439,28 +2439,28 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="B5" t="n">
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I5" t="n">
         <v>4</v>
@@ -2468,28 +2468,28 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B6" t="n">
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I6" t="n">
         <v>5</v>
@@ -2497,7 +2497,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B7" t="n">
         <v>0</v>
@@ -2506,19 +2506,19 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I7" t="n">
         <v>6</v>
@@ -2526,28 +2526,28 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B8" t="n">
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I8" t="n">
         <v>7</v>
@@ -2555,28 +2555,28 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B9" t="n">
         <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I9" t="n">
         <v>8</v>
@@ -2584,28 +2584,28 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B10" t="n">
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I10" t="n">
         <v>9</v>
@@ -2613,28 +2613,28 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B11" t="n">
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I11" t="n">
         <v>10</v>
@@ -2642,28 +2642,28 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I12" t="n">
         <v>11</v>
@@ -2671,28 +2671,28 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I13" t="n">
         <v>12</v>
@@ -2703,25 +2703,25 @@
         <v>0</v>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C14" t="n">
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
         <v>13</v>
@@ -2729,28 +2729,28 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I15" t="n">
         <v>14</v>
@@ -2758,25 +2758,25 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -2787,10 +2787,10 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
@@ -2802,10 +2802,10 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -2816,28 +2816,28 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I18" t="n">
         <v>17</v>
@@ -2848,22 +2848,22 @@
         <v>0</v>
       </c>
       <c r="B19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
@@ -2874,28 +2874,28 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C20" t="n">
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I20" t="n">
         <v>19</v>
@@ -2903,28 +2903,28 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21" t="n">
         <v>20</v>

</xml_diff>